<commit_message>
fix(unit07): correct formula references in lesson06 phase-2, phase-4, and ScenarioSwitchShowTell component
</commit_message>
<xml_diff>
--- a/bus-math-nextjs/public/resources/unit07-lesson06-student.xlsx
+++ b/bus-math-nextjs/public/resources/unit07-lesson06-student.xlsx
@@ -15,7 +15,22 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="SelectedScenario">'Inputs'!$B$4</definedName>
+    <definedName name="SelectedMethod">'Inputs'!$B$5</definedName>
+    <definedName name="SelectedKey">'Inputs'!$B$6</definedName>
+    <definedName name="UnitSellingPrice">'Inputs'!$B$8</definedName>
+    <definedName name="BeginningInventory">'Inputs'!$B$9</definedName>
+    <definedName name="GAFS">'Inputs'!$B$10</definedName>
+    <definedName name="SelectedUnitsSold">'Outputs'!$B$2</definedName>
+    <definedName name="SelectedCOGS">'Outputs'!$B$3</definedName>
+    <definedName name="SelectedEndingInventory">'Outputs'!$B$4</definedName>
+    <definedName name="Revenue">'KPI'!$B$2</definedName>
+    <definedName name="GrossMarginPct">'KPI'!$B$3</definedName>
+    <definedName name="AverageInventory">'KPI'!$B$4</definedName>
+    <definedName name="InventoryTurnover">'KPI'!$B$5</definedName>
+    <definedName name="DaysOnHand">'KPI'!$B$6</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -148,6 +163,34 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Drivers" displayName="Drivers" ref="A1:D4" headerRowCount="1">
+  <autoFilter ref="A1:D4"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Scenario"/>
+    <tableColumn id="2" name="UnitsSold"/>
+    <tableColumn id="3" name="DefaultMethod"/>
+    <tableColumn id="4" name="AsOfDate"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MethodSummary" displayName="MethodSummary" ref="A1:F10" headerRowCount="1">
+  <autoFilter ref="A1:F10"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Key"/>
+    <tableColumn id="2" name="Scenario"/>
+    <tableColumn id="3" name="Method"/>
+    <tableColumn id="4" name="COGS"/>
+    <tableColumn id="5" name="EndingInventory"/>
+    <tableColumn id="6" name="BalanceCheck"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -511,7 +554,6 @@
           <t>SelectedKey</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -544,6 +586,14 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Base,Stretch,Downside"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"FIFO,LIFO,Weighted Average"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -647,6 +697,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -715,9 +768,6 @@
           <t>FIFO</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -735,9 +785,6 @@
           <t>LIFO</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -755,9 +802,6 @@
           <t>Weighted Average</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -775,9 +819,6 @@
           <t>FIFO</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -795,9 +836,6 @@
           <t>LIFO</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -815,9 +853,6 @@
           <t>Weighted Average</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -835,9 +870,6 @@
           <t>FIFO</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -855,9 +887,6 @@
           <t>LIFO</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -875,12 +904,12 @@
           <t>Weighted Average</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -921,7 +950,6 @@
           <t>SelectedUnitsSold</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>XLOOKUP(SelectedScenario, Drivers[Scenario], Drivers[UnitsSold])</t>
@@ -934,7 +962,6 @@
           <t>SelectedCOGS</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>XLOOKUP(SelectedKey, MethodSummary[Key], MethodSummary[COGS])</t>
@@ -947,7 +974,6 @@
           <t>SelectedEndingInventory</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>XLOOKUP(SelectedKey, MethodSummary[Key], MethodSummary[EndingInventory])</t>
@@ -960,7 +986,6 @@
           <t>GAFS</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Input from Inputs</t>
@@ -1009,7 +1034,6 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>SelectedUnitsSold * UnitSellingPrice</t>
@@ -1022,7 +1046,6 @@
           <t>GrossMarginPct</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>(Revenue - SelectedCOGS) / Revenue</t>
@@ -1035,7 +1058,6 @@
           <t>AverageInventory</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>(BeginningInventory + SelectedEndingInventory) / 2</t>
@@ -1048,7 +1070,6 @@
           <t>InventoryTurnover</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>SelectedCOGS / AverageInventory</t>
@@ -1061,7 +1082,6 @@
           <t>DaysOnHand</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>365 / InventoryTurnover</t>
@@ -1110,10 +1130,9 @@
           <t>GAFS Balance</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IF(ABS((SelectedCOGS+SelectedEI)-GAFS)&lt;0.01,"Balanced","Check")</t>
+          <t>IF(ABS((SelectedCOGS+SelectedEndingInventory)-GAFS)&lt;0.01,"Balanced","Check")</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1142,6 @@
           <t>SelectedKey Found</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>IFNA(XLOOKUP(SelectedKey, MethodSummary[Key], MethodSummary[COGS]),"Missing Key")</t>
@@ -1136,7 +1154,6 @@
           <t>Units Sold Valid</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>IF(SelectedUnitsSold&gt;0,"OK","Check Drivers")</t>
@@ -1185,7 +1202,6 @@
           <t>Scenario</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Inputs!B4</t>
@@ -1198,7 +1214,6 @@
           <t>Method</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Inputs!B5</t>
@@ -1211,7 +1226,6 @@
           <t>COGS</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Outputs!B3</t>
@@ -1224,7 +1238,6 @@
           <t>Ending Inventory</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Outputs!B4</t>
@@ -1237,7 +1250,6 @@
           <t>Turnover</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>KPI!B5</t>
@@ -1250,7 +1262,6 @@
           <t>Days on Hand</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>KPI!B6</t>
@@ -1263,7 +1274,6 @@
           <t>Gross Margin %</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>KPI!B3</t>
@@ -1276,7 +1286,6 @@
           <t>Check Status</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Checks!B2</t>

</xml_diff>